<commit_message>
feat: update paper changes
</commit_message>
<xml_diff>
--- a/Papers.xlsx
+++ b/Papers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GithubProjects\prethesis-experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BEE5D82-18AB-41DD-ACB9-AA592A2E62EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AED4249-CE2D-4424-807F-85BB68675E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{92B0260C-7ECB-4F59-B7C2-732AB9F78D30}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -55,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>Paper Name</t>
   </si>
@@ -166,13 +165,22 @@
   </si>
   <si>
     <t>A survey on deep learning for textual emotion analysis in social networks</t>
+  </si>
+  <si>
+    <t>https://comengapp.unsri.ac.id/index.php/comengapp/article/view/494</t>
+  </si>
+  <si>
+    <t>Emotion Classification in Indonesian Text Using IndoBERT</t>
+  </si>
+  <si>
+    <t>Using indobert for emotion classification</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -196,6 +204,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="21"/>
+      <color rgb="FF333333"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -218,7 +233,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -244,15 +259,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -283,6 +298,9 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -305,16 +323,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{949D47CF-C519-405A-AE08-3D0DBECB1FBE}" name="Table1" displayName="Table1" ref="B2:E14" totalsRowShown="0" headerRowDxfId="5" dataDxfId="0">
-  <autoFilter ref="B2:E14" xr:uid="{949D47CF-C519-405A-AE08-3D0DBECB1FBE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{949D47CF-C519-405A-AE08-3D0DBECB1FBE}" name="Table1" displayName="Table1" ref="B2:E15" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="B2:E15" xr:uid="{949D47CF-C519-405A-AE08-3D0DBECB1FBE}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:E4">
     <sortCondition ref="E2:E4"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{60BD311D-5397-421D-8968-AA3580F42936}" name="Paper Name" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{C656A76D-5779-4852-BFEF-9F5F7C1AA439}" name="Link" dataDxfId="3" dataCellStyle="Hyperlink"/>
-    <tableColumn id="3" xr3:uid="{38C81947-8B9B-4D6B-801C-88F942918980}" name="Description" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{B00545BA-C939-4B08-A3E6-3D3A467C1A47}" name="Date Added" dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{60BD311D-5397-421D-8968-AA3580F42936}" name="Paper Name" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{C656A76D-5779-4852-BFEF-9F5F7C1AA439}" name="Link" dataDxfId="2" dataCellStyle="Hyperlink"/>
+    <tableColumn id="3" xr3:uid="{38C81947-8B9B-4D6B-801C-88F942918980}" name="Description" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{B00545BA-C939-4B08-A3E6-3D3A467C1A47}" name="Date Added" dataDxfId="0">
       <calculatedColumnFormula>NOW()</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -684,7 +702,7 @@
       </c>
       <c r="E3" s="7">
         <f t="shared" ref="E3:E13" ca="1" si="0">NOW()</f>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="4" spans="2:5" ht="30" x14ac:dyDescent="0.25">
@@ -699,7 +717,7 @@
       </c>
       <c r="E4" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="30" x14ac:dyDescent="0.25">
@@ -714,7 +732,7 @@
       </c>
       <c r="E5" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="45" x14ac:dyDescent="0.25">
@@ -729,7 +747,7 @@
       </c>
       <c r="E6" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
@@ -744,7 +762,7 @@
       </c>
       <c r="E7" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="30" x14ac:dyDescent="0.25">
@@ -759,7 +777,7 @@
       </c>
       <c r="E8" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="45" x14ac:dyDescent="0.25">
@@ -774,7 +792,7 @@
       </c>
       <c r="E9" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="30" x14ac:dyDescent="0.25">
@@ -789,7 +807,7 @@
       </c>
       <c r="E10" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="45" x14ac:dyDescent="0.25">
@@ -804,7 +822,7 @@
       </c>
       <c r="E11" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="105" x14ac:dyDescent="0.25">
@@ -817,7 +835,7 @@
       <c r="D12" s="6"/>
       <c r="E12" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="45" x14ac:dyDescent="0.25">
@@ -830,7 +848,7 @@
       <c r="D13" s="6"/>
       <c r="E13" s="7">
         <f t="shared" ca="1" si="0"/>
-        <v>45728.638656944444</v>
+        <v>45730.571695949075</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="409.5" x14ac:dyDescent="0.25">
@@ -843,14 +861,23 @@
       <c r="D14" s="6"/>
       <c r="E14" s="7">
         <f ca="1">NOW()</f>
-        <v>45728.638656944444</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="3"/>
+        <v>45730.571695949075</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="7">
+        <f ca="1">NOW()</f>
+        <v>45730.571695949075</v>
+      </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>

</xml_diff>